<commit_message>
feat(antelope): AI网页选值流程 + common.py公共工具重构 + fr_dress批次数据
</commit_message>
<xml_diff>
--- a/antelope/xlsm/8.18v1.xlsx
+++ b/antelope/xlsm/8.18v1.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FW20260325\besskyproject\dealExcel_refactoring\antelope\xlsm\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\jetbrains_projects\pycharmProjects\Tools-For-Fuck-Work\antelope\xlsm\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12375"/>
+    <workbookView windowWidth="27945" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet0" sheetId="1" r:id="rId1"/>
@@ -2239,7 +2239,15 @@
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="18">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2433,25 +2441,25 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="totalRow" dxfId="5"/>
+      <tableStyleElement type="firstColumn" dxfId="4"/>
+      <tableStyleElement type="lastColumn" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="1"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="17"/>
+      <tableStyleElement type="totalRow" dxfId="16"/>
+      <tableStyleElement type="firstRowStripe" dxfId="15"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="14"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="13"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="11"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="10"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="9"/>
+      <tableStyleElement type="pageFieldValues" dxfId="8"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -2881,7 +2889,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="13296900" y="635000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2920,7 +2928,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="26108660" y="635000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2959,7 +2967,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="27538680" y="635000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2998,7 +3006,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="28910280" y="635000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3037,7 +3045,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="30281880" y="635000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3075,8 +3083,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13296900" y="4445000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="13296900" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3114,8 +3122,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="26108660" y="4445000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="26108660" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3153,8 +3161,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="27538680" y="4445000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="27538680" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3192,8 +3200,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="30281880" y="4445000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="30281880" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3231,8 +3239,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13296900" y="8255000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="13296900" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3270,8 +3278,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="26108660" y="8255000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="26108660" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3309,8 +3317,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="27538680" y="8255000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="27538680" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3348,8 +3356,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="30281880" y="8255000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="30281880" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3387,8 +3395,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="31653480" y="8255000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="31653480" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3426,8 +3434,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="33025080" y="8255000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="33025080" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3465,8 +3473,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="34396680" y="8255000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="34396680" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3504,8 +3512,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="35768280" y="8255000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="35768280" y="635000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3543,7 +3551,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13296900" y="12065000"/>
+          <a:off x="13296900" y="635000"/>
           <a:ext cx="645160" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3582,7 +3590,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="26108660" y="12065000"/>
+          <a:off x="26108660" y="635000"/>
           <a:ext cx="645160" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3621,7 +3629,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="27538680" y="12065000"/>
+          <a:off x="27538680" y="635000"/>
           <a:ext cx="645160" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3660,7 +3668,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28910280" y="12065000"/>
+          <a:off x="28910280" y="635000"/>
           <a:ext cx="645160" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3699,7 +3707,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="30281880" y="12065000"/>
+          <a:off x="30281880" y="635000"/>
           <a:ext cx="645160" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3738,7 +3746,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="31653480" y="12065000"/>
+          <a:off x="31653480" y="635000"/>
           <a:ext cx="645160" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3777,7 +3785,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="33025080" y="12065000"/>
+          <a:off x="33025080" y="635000"/>
           <a:ext cx="645160" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3816,7 +3824,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="34396680" y="12065000"/>
+          <a:off x="34396680" y="635000"/>
           <a:ext cx="645160" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3855,7 +3863,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="35768280" y="12065000"/>
+          <a:off x="35768280" y="635000"/>
           <a:ext cx="645160" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3894,7 +3902,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="37139880" y="12065000"/>
+          <a:off x="37139880" y="635000"/>
           <a:ext cx="645160" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3933,8 +3941,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13296900" y="12700000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="13296900" y="1270000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3972,8 +3980,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="26108660" y="12700000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="26108660" y="1270000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4011,8 +4019,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="27538680" y="12700000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="27538680" y="1270000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4050,8 +4058,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28910280" y="12700000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="28910280" y="1270000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4089,8 +4097,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="30281880" y="12700000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="30281880" y="1270000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4128,8 +4136,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="31653480" y="12700000"/>
-          <a:ext cx="645160" cy="571500"/>
+          <a:off x="31653480" y="1270000"/>
+          <a:ext cx="645160" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4401,7 +4409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:BO26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
@@ -4436,7 +4444,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="4">
-        <f>LEN(E1)</f>
+        <f t="shared" ref="F1:F19" si="0">LEN(E1)</f>
         <v>114</v>
       </c>
       <c r="G1" s="4"/>
@@ -4586,7 +4594,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" ht="50" customHeight="1" spans="1:67">
+    <row r="2" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A2" s="4" t="s">
         <v>34</v>
       </c>
@@ -4597,15 +4605,15 @@
         <v>1</v>
       </c>
       <c r="D2" s="4" t="str">
-        <f t="shared" ref="D2:D31" si="0">D1</f>
+        <f t="shared" ref="D2:D31" si="1">D1</f>
         <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
       </c>
       <c r="E2" s="4" t="str">
-        <f t="shared" ref="E2:E31" si="1">E1</f>
+        <f t="shared" ref="E2:E31" si="2">E1</f>
         <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
       </c>
       <c r="F2" s="4">
-        <f>LEN(E2)</f>
+        <f t="shared" si="0"/>
         <v>114</v>
       </c>
       <c r="G2" s="4"/>
@@ -4714,67 +4722,67 @@
         <v>26.32</v>
       </c>
       <c r="AY2" t="str">
-        <f t="shared" ref="AY2:AY31" si="2">AY1</f>
+        <f t="shared" ref="AY2:AY31" si="3">AY1</f>
         <v>Sans col</v>
       </c>
       <c r="AZ2" t="str">
-        <f t="shared" ref="AZ2:AZ31" si="3">AZ1</f>
+        <f t="shared" ref="AZ2:AZ31" si="4">AZ1</f>
         <v>Décontracté</v>
       </c>
       <c r="BA2" t="str">
-        <f t="shared" ref="BA2:BA31" si="4">BA1</f>
+        <f t="shared" ref="BA2:BA31" si="5">BA1</f>
         <v>Minimaliste</v>
       </c>
       <c r="BB2" t="str">
-        <f t="shared" ref="BB2:BB31" si="5">BB1</f>
+        <f t="shared" ref="BB2:BB31" si="6">BB1</f>
         <v>Chemise</v>
       </c>
       <c r="BC2" t="str">
-        <f t="shared" ref="BC2:BC31" si="6">BC1</f>
+        <f t="shared" ref="BC2:BC31" si="7">BC1</f>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD2" t="str">
-        <f t="shared" ref="BD2:BD31" si="7">BD1</f>
+        <f t="shared" ref="BD2:BD31" si="8">BD1</f>
         <v>Plaine</v>
       </c>
       <c r="BE2" t="str">
-        <f t="shared" ref="BE2:BE31" si="8">BE1</f>
+        <f t="shared" ref="BE2:BE31" si="9">BE1</f>
         <v>À capuche</v>
       </c>
       <c r="BG2" t="str">
-        <f t="shared" ref="BG2:BG31" si="9">BG1</f>
+        <f t="shared" ref="BG2:BG31" si="10">BG1</f>
         <v>Manches longues</v>
       </c>
       <c r="BH2" t="str">
-        <f t="shared" ref="BH2:BH31" si="10">BH1</f>
+        <f t="shared" ref="BH2:BH31" si="11">BH1</f>
         <v>Manchette</v>
       </c>
       <c r="BI2" t="str">
-        <f t="shared" ref="BI2:BI31" si="11">BI1</f>
+        <f t="shared" ref="BI2:BI31" si="12">BI1</f>
         <v>Bouton</v>
       </c>
       <c r="BK2" t="str">
-        <f t="shared" ref="BK2:BK31" si="12">BK1</f>
+        <f t="shared" ref="BK2:BK31" si="13">BK1</f>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL2" t="str">
-        <f t="shared" ref="BL2:BL31" si="13">BL1</f>
+        <f t="shared" ref="BL2:BL31" si="14">BL1</f>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM2" t="str">
-        <f t="shared" ref="BM2:BM31" si="14">BM1</f>
+        <f t="shared" ref="BM2:BM31" si="15">BM1</f>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN2" t="str">
-        <f t="shared" ref="BN2:BN31" si="15">BN1</f>
+        <f t="shared" ref="BN2:BN31" si="16">BN1</f>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO2" t="str">
-        <f t="shared" ref="BO2:BO31" si="16">BO1</f>
+        <f t="shared" ref="BO2:BO31" si="17">BO1</f>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="3" ht="50" customHeight="1" spans="1:67">
+    <row r="3" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A3" s="4" t="s">
         <v>46</v>
       </c>
@@ -4785,15 +4793,15 @@
         <v>1</v>
       </c>
       <c r="D3" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E3" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F3" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E3" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F3" s="4">
-        <f>LEN(E3)</f>
         <v>114</v>
       </c>
       <c r="G3" s="4"/>
@@ -4902,67 +4910,67 @@
         <v>26.34</v>
       </c>
       <c r="AY3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB3" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC3" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD3" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE3" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG3" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH3" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI3" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK3" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL3" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM3" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN3" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO3" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="4" ht="50" customHeight="1" spans="1:67">
+    <row r="4" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A4" s="4" t="s">
         <v>56</v>
       </c>
@@ -4973,15 +4981,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E4" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F4" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E4" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F4" s="4">
-        <f>LEN(E4)</f>
         <v>114</v>
       </c>
       <c r="G4" s="4"/>
@@ -5090,67 +5098,67 @@
         <v>26.34</v>
       </c>
       <c r="AY4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG4" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH4" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI4" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL4" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM4" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN4" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO4" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="5" ht="50" customHeight="1" spans="1:67">
+    <row r="5" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A5" s="4" t="s">
         <v>66</v>
       </c>
@@ -5161,15 +5169,15 @@
         <v>1</v>
       </c>
       <c r="D5" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E5" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F5" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E5" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F5" s="4">
-        <f>LEN(E5)</f>
         <v>114</v>
       </c>
       <c r="G5" s="4"/>
@@ -5278,67 +5286,67 @@
         <v>26.42</v>
       </c>
       <c r="AY5" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ5" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC5" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD5" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE5" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG5" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH5" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI5" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK5" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL5" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM5" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN5" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO5" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="6" ht="50" customHeight="1" spans="1:67">
+    <row r="6" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A6" s="4" t="s">
         <v>76</v>
       </c>
@@ -5349,15 +5357,15 @@
         <v>1</v>
       </c>
       <c r="D6" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E6" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F6" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E6" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F6" s="4">
-        <f>LEN(E6)</f>
         <v>114</v>
       </c>
       <c r="G6" s="4"/>
@@ -5466,67 +5474,67 @@
         <v>26.24</v>
       </c>
       <c r="AY6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB6" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC6" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG6" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH6" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI6" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK6" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL6" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM6" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN6" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO6" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="7" ht="50" customHeight="1" spans="1:67">
+    <row r="7" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A7" s="4" t="s">
         <v>86</v>
       </c>
@@ -5537,15 +5545,15 @@
         <v>1</v>
       </c>
       <c r="D7" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E7" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F7" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E7" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F7" s="4">
-        <f>LEN(E7)</f>
         <v>114</v>
       </c>
       <c r="G7" s="4"/>
@@ -5654,67 +5662,67 @@
         <v>26.33</v>
       </c>
       <c r="AY7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ7" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA7" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD7" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG7" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH7" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI7" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK7" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL7" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM7" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN7" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO7" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="8" ht="50" customHeight="1" spans="1:67">
+    <row r="8" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A8" s="4" t="s">
         <v>96</v>
       </c>
@@ -5725,15 +5733,15 @@
         <v>1</v>
       </c>
       <c r="D8" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E8" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F8" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E8" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F8" s="4">
-        <f>LEN(E8)</f>
         <v>114</v>
       </c>
       <c r="G8" s="4"/>
@@ -5842,67 +5850,67 @@
         <v>26.06</v>
       </c>
       <c r="AY8" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ8" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB8" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC8" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD8" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE8" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG8" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH8" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI8" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK8" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL8" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM8" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN8" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO8" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="9" ht="50" customHeight="1" spans="1:67">
+    <row r="9" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A9" s="4" t="s">
         <v>107</v>
       </c>
@@ -5913,15 +5921,15 @@
         <v>1</v>
       </c>
       <c r="D9" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E9" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F9" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E9" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F9" s="4">
-        <f>LEN(E9)</f>
         <v>114</v>
       </c>
       <c r="G9" s="4"/>
@@ -6030,67 +6038,67 @@
         <v>26.23</v>
       </c>
       <c r="AY9" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ9" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA9" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB9" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC9" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD9" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE9" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG9" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH9" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI9" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK9" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL9" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM9" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN9" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO9" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="10" ht="50" customHeight="1" spans="1:67">
+    <row r="10" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A10" s="4" t="s">
         <v>116</v>
       </c>
@@ -6101,15 +6109,15 @@
         <v>1</v>
       </c>
       <c r="D10" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E10" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F10" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E10" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F10" s="4">
-        <f>LEN(E10)</f>
         <v>114</v>
       </c>
       <c r="G10" s="4"/>
@@ -6218,67 +6226,67 @@
         <v>26.69</v>
       </c>
       <c r="AY10" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ10" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA10" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB10" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC10" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD10" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE10" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG10" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH10" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI10" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK10" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL10" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM10" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN10" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO10" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="11" ht="50" customHeight="1" spans="1:67">
+    <row r="11" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A11" s="4" t="s">
         <v>125</v>
       </c>
@@ -6289,15 +6297,15 @@
         <v>1</v>
       </c>
       <c r="D11" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E11" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F11" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E11" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F11" s="4">
-        <f>LEN(E11)</f>
         <v>114</v>
       </c>
       <c r="G11" s="4"/>
@@ -6406,67 +6414,67 @@
         <v>26.22</v>
       </c>
       <c r="AY11" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ11" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA11" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB11" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC11" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD11" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE11" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG11" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH11" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI11" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK11" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL11" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM11" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN11" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO11" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="12" ht="50" customHeight="1" spans="1:67">
+    <row r="12" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A12" s="4" t="s">
         <v>134</v>
       </c>
@@ -6477,15 +6485,15 @@
         <v>1</v>
       </c>
       <c r="D12" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E12" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F12" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E12" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F12" s="4">
-        <f>LEN(E12)</f>
         <v>114</v>
       </c>
       <c r="G12" s="4"/>
@@ -6594,67 +6602,67 @@
         <v>26.06</v>
       </c>
       <c r="AY12" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ12" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA12" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB12" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC12" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD12" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE12" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG12" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH12" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI12" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK12" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL12" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM12" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN12" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO12" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="13" ht="50" customHeight="1" spans="1:67">
+    <row r="13" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A13" s="4" t="s">
         <v>143</v>
       </c>
@@ -6665,15 +6673,15 @@
         <v>1</v>
       </c>
       <c r="D13" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E13" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F13" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E13" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F13" s="4">
-        <f>LEN(E13)</f>
         <v>114</v>
       </c>
       <c r="G13" s="4"/>
@@ -6782,67 +6790,67 @@
         <v>26.09</v>
       </c>
       <c r="AY13" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ13" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA13" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB13" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC13" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD13" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE13" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG13" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH13" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI13" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK13" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL13" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM13" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN13" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO13" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="14" ht="50" customHeight="1" spans="1:67">
+    <row r="14" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A14" s="4" t="s">
         <v>152</v>
       </c>
@@ -6853,15 +6861,15 @@
         <v>1</v>
       </c>
       <c r="D14" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E14" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F14" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E14" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F14" s="4">
-        <f>LEN(E14)</f>
         <v>114</v>
       </c>
       <c r="G14" s="4"/>
@@ -6970,67 +6978,67 @@
         <v>26.22</v>
       </c>
       <c r="AY14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA14" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB14" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE14" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG14" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH14" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI14" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK14" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL14" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM14" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN14" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO14" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="15" ht="50" customHeight="1" spans="1:67">
+    <row r="15" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A15" s="4" t="s">
         <v>165</v>
       </c>
@@ -7041,15 +7049,15 @@
         <v>1</v>
       </c>
       <c r="D15" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E15" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F15" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E15" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F15" s="4">
-        <f>LEN(E15)</f>
         <v>114</v>
       </c>
       <c r="G15" s="4"/>
@@ -7158,67 +7166,67 @@
         <v>26.36</v>
       </c>
       <c r="AY15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA15" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG15" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH15" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI15" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK15" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL15" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM15" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN15" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO15" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="16" ht="50" customHeight="1" spans="1:67">
+    <row r="16" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A16" s="4" t="s">
         <v>178</v>
       </c>
@@ -7229,15 +7237,15 @@
         <v>1</v>
       </c>
       <c r="D16" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E16" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F16" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E16" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F16" s="4">
-        <f>LEN(E16)</f>
         <v>114</v>
       </c>
       <c r="G16" s="4"/>
@@ -7346,67 +7354,67 @@
         <v>26.21</v>
       </c>
       <c r="AY16" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ16" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA16" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB16" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC16" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD16" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE16" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG16" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH16" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI16" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK16" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL16" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM16" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN16" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO16" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="17" ht="50" customHeight="1" spans="1:67">
+    <row r="17" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A17" s="4" t="s">
         <v>191</v>
       </c>
@@ -7417,15 +7425,15 @@
         <v>1</v>
       </c>
       <c r="D17" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E17" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F17" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E17" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F17" s="4">
-        <f>LEN(E17)</f>
         <v>114</v>
       </c>
       <c r="G17" s="4"/>
@@ -7534,67 +7542,67 @@
         <v>26.23</v>
       </c>
       <c r="AY17" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ17" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA17" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB17" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC17" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD17" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE17" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG17" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH17" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI17" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK17" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL17" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM17" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN17" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO17" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="18" ht="50" customHeight="1" spans="1:67">
+    <row r="18" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A18" s="4" t="s">
         <v>203</v>
       </c>
@@ -7605,15 +7613,15 @@
         <v>1</v>
       </c>
       <c r="D18" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E18" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F18" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E18" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F18" s="4">
-        <f>LEN(E18)</f>
         <v>114</v>
       </c>
       <c r="G18" s="4"/>
@@ -7722,67 +7730,67 @@
         <v>26.16</v>
       </c>
       <c r="AY18" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA18" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC18" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE18" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH18" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI18" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK18" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL18" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM18" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN18" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO18" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
-    <row r="19" ht="50" customHeight="1" spans="1:67">
+    <row r="19" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A19" s="4" t="s">
         <v>216</v>
       </c>
@@ -7793,15 +7801,15 @@
         <v>1</v>
       </c>
       <c r="D19" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
+      </c>
+      <c r="E19" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
+      </c>
+      <c r="F19" s="4">
         <f t="shared" si="0"/>
-        <v>Cardigan Homme Capuche Lin Manches Longues Ample Cintré</v>
-      </c>
-      <c r="E19" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Coton Fin Respirant Anti-UV Cordon de Serrage Demi-Ouverture Ourlet Courbe Vacances Décontracté Cardigan Essentiel</v>
-      </c>
-      <c r="F19" s="4">
-        <f>LEN(E19)</f>
         <v>114</v>
       </c>
       <c r="G19" s="4"/>
@@ -7910,63 +7918,63 @@
         <v>26.09</v>
       </c>
       <c r="AY19" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Sans col</v>
       </c>
       <c r="AZ19" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>Décontracté</v>
       </c>
       <c r="BA19" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Minimaliste</v>
       </c>
       <c r="BB19" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Chemise</v>
       </c>
       <c r="BC19" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Surdimensionnée</v>
       </c>
       <c r="BD19" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>Plaine</v>
       </c>
       <c r="BE19" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>À capuche</v>
       </c>
       <c r="BG19" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>Manches longues</v>
       </c>
       <c r="BH19" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>Manchette</v>
       </c>
       <c r="BI19" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>Bouton</v>
       </c>
       <c r="BK19" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>Tissu respirant : profitez d’un confort optimal au quotidien, car nos chemises pour homme sont confectionnées dans un tissu de qualité supérieure, très respirant, qui vous garantit un confort optimal.</v>
       </c>
       <c r="BL19" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>Design classique et tendance : cette chemise intemporelle, au style très tendance, allie élégance et charme décontracté, ce qui la rend idéale pour toutes les occasions décontractées.</v>
       </c>
       <c r="BM19" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>Polyvalente et adaptée à toutes les occasions : que ce soit pour aller à la plage, participer à un barbecue estival ou simplement vous détendre chez vous, cette chemise en lin à manches longues pour homme est le choix idéal pour créer un look décontracté.</v>
       </c>
       <c r="BN19" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>Facile à assortir : associez cette chemise unie classique à un short, un pantalon kaki ou un jean pour créer un look raffiné sans effort, qui s'adapte aussi bien à la journée qu'à la soirée.</v>
       </c>
       <c r="BO19" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>Résistante et facile d’entretien : confectionnée avec un savoir-faire exceptionnel, cette chemise d’été est non seulement élégante et raffinée, mais elle est également lavable en machine et facile à entretenir, ce qui garantit qu’elle restera un incontournable de votre garde-robe pendant de nombreuses années.</v>
       </c>
     </row>
@@ -7987,7 +7995,7 @@
         <v>231</v>
       </c>
       <c r="F20" s="4">
-        <f t="shared" ref="F20:F52" si="17">LEN(E20)</f>
+        <f t="shared" ref="F20:F52" si="18">LEN(E20)</f>
         <v>105</v>
       </c>
       <c r="G20" s="4"/>
@@ -8137,7 +8145,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="21" ht="50" customHeight="1" spans="1:67">
+    <row r="21" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A21" s="4" t="s">
         <v>254</v>
       </c>
@@ -8148,15 +8156,15 @@
         <v>229</v>
       </c>
       <c r="D21" s="4" t="str">
-        <f t="shared" ref="D21:D50" si="18">D20</f>
+        <f t="shared" ref="D21:D50" si="19">D20</f>
         <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
       </c>
       <c r="E21" s="4" t="str">
-        <f t="shared" ref="E21:E50" si="19">E20</f>
+        <f t="shared" ref="E21:E50" si="20">E20</f>
         <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
       </c>
       <c r="F21" s="4">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>105</v>
       </c>
       <c r="G21" s="4"/>
@@ -8265,67 +8273,67 @@
         <v>23.26</v>
       </c>
       <c r="AY21" t="str">
-        <f t="shared" ref="AY21:AY50" si="20">AY20</f>
+        <f t="shared" ref="AY21:AY50" si="21">AY20</f>
         <v>Col rabattu</v>
       </c>
       <c r="AZ21" t="str">
-        <f t="shared" ref="AZ21:AZ50" si="21">AZ20</f>
+        <f t="shared" ref="AZ21:AZ50" si="22">AZ20</f>
         <v>Décontracté</v>
       </c>
       <c r="BA21" t="str">
-        <f t="shared" ref="BA21:BA50" si="22">BA20</f>
+        <f t="shared" ref="BA21:BA50" si="23">BA20</f>
         <v>Occidental</v>
       </c>
       <c r="BB21" t="str">
-        <f t="shared" ref="BB21:BB50" si="23">BB20</f>
+        <f t="shared" ref="BB21:BB50" si="24">BB20</f>
         <v>Chemise</v>
       </c>
       <c r="BC21" t="str">
-        <f t="shared" ref="BC21:BC50" si="24">BC20</f>
+        <f t="shared" ref="BC21:BC50" si="25">BC20</f>
         <v>Régulier</v>
       </c>
       <c r="BD21" t="str">
-        <f t="shared" ref="BD21:BD50" si="25">BD20</f>
+        <f t="shared" ref="BD21:BD50" si="26">BD20</f>
         <v>Plaine</v>
       </c>
       <c r="BE21" t="str">
-        <f t="shared" ref="BE21:BE50" si="26">BE20</f>
+        <f t="shared" ref="BE21:BE50" si="27">BE20</f>
         <v>Col cranté</v>
       </c>
       <c r="BG21" t="str">
-        <f t="shared" ref="BG21:BG50" si="27">BG20</f>
+        <f t="shared" ref="BG21:BG50" si="28">BG20</f>
         <v>Manches longues</v>
       </c>
       <c r="BH21" t="str">
-        <f t="shared" ref="BH21:BH50" si="28">BH20</f>
+        <f t="shared" ref="BH21:BH50" si="29">BH20</f>
         <v>Manchette</v>
       </c>
       <c r="BI21" t="str">
-        <f t="shared" ref="BI21:BI50" si="29">BI20</f>
+        <f t="shared" ref="BI21:BI50" si="30">BI20</f>
         <v>Bouton</v>
       </c>
       <c r="BK21" t="str">
-        <f t="shared" ref="BK21:BK50" si="30">BK20</f>
+        <f t="shared" ref="BK21:BK50" si="31">BK20</f>
         <v>Tissu ultra-légèrement aéré : grâce à une sélection de matières premières nobles, nos chemises homme offrent une respirabilité exceptionnelle qui vous enveloppe d’une sensation de fraîcheur tout au long de la journée.</v>
       </c>
       <c r="BL21" t="str">
-        <f t="shared" ref="BL21:BL50" si="31">BL20</f>
+        <f t="shared" ref="BL21:BL50" si="32">BL20</f>
         <v>Coupe moderne et intemporelle : ce modèle au design épuré mêle avec subtilité l’esprit classique et une touche contemporaine, pour un rendu aussi chic que décontracté, parfait pour vos journées estivales.</v>
       </c>
       <c r="BM21" t="str">
-        <f t="shared" ref="BM21:BM50" si="32">BM20</f>
+        <f t="shared" ref="BM21:BM50" si="33">BM20</f>
         <v>Adaptée à toutes les situations : que vous flâniez en bord de mer, que vous participiez à un pique-nique entre amis ou que vous profitiez d’un moment de farniente à la maison, cette chemise en lin à manches longues s’impose comme la pièce maîtresse de vos tenues décontractées.</v>
       </c>
       <c r="BN21" t="str">
-        <f t="shared" ref="BN21:BN50" si="33">BN20</f>
+        <f t="shared" ref="BN21:BN50" si="34">BN20</f>
         <v>Associations faciles et infinies : portez-la avec un bermuda, un pantalon en toile ou un jean brut, et vous obtiendrez en un clin d’œil une allure élégante et naturelle, qui passe sans effort de la lumière du jour aux soirées douces.</v>
       </c>
       <c r="BO21" t="str">
-        <f t="shared" ref="BO21:BO50" si="34">BO20</f>
+        <f t="shared" ref="BO21:BO50" si="35">BO20</f>
         <v>Solidité et entretien simplifié : confectionnée selon un savoir-faire rigoureux, cette chemise d’été allie esthétique raffinée et praticité – elle supporte parfaitement le lavage en machine et conserve son éclat saison après saison, devenant vite un indispensable de votre dressing.</v>
       </c>
     </row>
-    <row r="22" ht="50" customHeight="1" spans="1:67">
+    <row r="22" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A22" s="4" t="s">
         <v>266</v>
       </c>
@@ -8336,15 +8344,15 @@
         <v>229</v>
       </c>
       <c r="D22" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
+      </c>
+      <c r="E22" s="4" t="str">
+        <f t="shared" si="20"/>
+        <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
+      </c>
+      <c r="F22" s="4">
         <f t="shared" si="18"/>
-        <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
-      </c>
-      <c r="E22" s="4" t="str">
-        <f t="shared" si="19"/>
-        <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
-      </c>
-      <c r="F22" s="4">
-        <f t="shared" si="17"/>
         <v>105</v>
       </c>
       <c r="G22" s="4"/>
@@ -8453,67 +8461,67 @@
         <v>24.94</v>
       </c>
       <c r="AY22" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>Col rabattu</v>
       </c>
       <c r="AZ22" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>Décontracté</v>
       </c>
       <c r="BA22" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>Occidental</v>
       </c>
       <c r="BB22" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>Chemise</v>
       </c>
       <c r="BC22" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>Régulier</v>
       </c>
       <c r="BD22" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>Plaine</v>
       </c>
       <c r="BE22" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>Col cranté</v>
       </c>
       <c r="BG22" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>Manches longues</v>
       </c>
       <c r="BH22" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>Manchette</v>
       </c>
       <c r="BI22" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>Bouton</v>
       </c>
       <c r="BK22" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>Tissu ultra-légèrement aéré : grâce à une sélection de matières premières nobles, nos chemises homme offrent une respirabilité exceptionnelle qui vous enveloppe d’une sensation de fraîcheur tout au long de la journée.</v>
       </c>
       <c r="BL22" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>Coupe moderne et intemporelle : ce modèle au design épuré mêle avec subtilité l’esprit classique et une touche contemporaine, pour un rendu aussi chic que décontracté, parfait pour vos journées estivales.</v>
       </c>
       <c r="BM22" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>Adaptée à toutes les situations : que vous flâniez en bord de mer, que vous participiez à un pique-nique entre amis ou que vous profitiez d’un moment de farniente à la maison, cette chemise en lin à manches longues s’impose comme la pièce maîtresse de vos tenues décontractées.</v>
       </c>
       <c r="BN22" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>Associations faciles et infinies : portez-la avec un bermuda, un pantalon en toile ou un jean brut, et vous obtiendrez en un clin d’œil une allure élégante et naturelle, qui passe sans effort de la lumière du jour aux soirées douces.</v>
       </c>
       <c r="BO22" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>Solidité et entretien simplifié : confectionnée selon un savoir-faire rigoureux, cette chemise d’été allie esthétique raffinée et praticité – elle supporte parfaitement le lavage en machine et conserve son éclat saison après saison, devenant vite un indispensable de votre dressing.</v>
       </c>
     </row>
-    <row r="23" ht="50" customHeight="1" spans="1:67">
+    <row r="23" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A23" s="4" t="s">
         <v>276</v>
       </c>
@@ -8524,15 +8532,15 @@
         <v>229</v>
       </c>
       <c r="D23" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
+      </c>
+      <c r="E23" s="4" t="str">
+        <f t="shared" si="20"/>
+        <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
+      </c>
+      <c r="F23" s="4">
         <f t="shared" si="18"/>
-        <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
-      </c>
-      <c r="E23" s="4" t="str">
-        <f t="shared" si="19"/>
-        <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
-      </c>
-      <c r="F23" s="4">
-        <f t="shared" si="17"/>
         <v>105</v>
       </c>
       <c r="G23" s="4"/>
@@ -8641,67 +8649,67 @@
         <v>25.02</v>
       </c>
       <c r="AY23" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>Col rabattu</v>
       </c>
       <c r="AZ23" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>Décontracté</v>
       </c>
       <c r="BA23" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>Occidental</v>
       </c>
       <c r="BB23" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>Chemise</v>
       </c>
       <c r="BC23" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>Régulier</v>
       </c>
       <c r="BD23" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>Plaine</v>
       </c>
       <c r="BE23" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>Col cranté</v>
       </c>
       <c r="BG23" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>Manches longues</v>
       </c>
       <c r="BH23" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>Manchette</v>
       </c>
       <c r="BI23" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>Bouton</v>
       </c>
       <c r="BK23" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>Tissu ultra-légèrement aéré : grâce à une sélection de matières premières nobles, nos chemises homme offrent une respirabilité exceptionnelle qui vous enveloppe d’une sensation de fraîcheur tout au long de la journée.</v>
       </c>
       <c r="BL23" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>Coupe moderne et intemporelle : ce modèle au design épuré mêle avec subtilité l’esprit classique et une touche contemporaine, pour un rendu aussi chic que décontracté, parfait pour vos journées estivales.</v>
       </c>
       <c r="BM23" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>Adaptée à toutes les situations : que vous flâniez en bord de mer, que vous participiez à un pique-nique entre amis ou que vous profitiez d’un moment de farniente à la maison, cette chemise en lin à manches longues s’impose comme la pièce maîtresse de vos tenues décontractées.</v>
       </c>
       <c r="BN23" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>Associations faciles et infinies : portez-la avec un bermuda, un pantalon en toile ou un jean brut, et vous obtiendrez en un clin d’œil une allure élégante et naturelle, qui passe sans effort de la lumière du jour aux soirées douces.</v>
       </c>
       <c r="BO23" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>Solidité et entretien simplifié : confectionnée selon un savoir-faire rigoureux, cette chemise d’été allie esthétique raffinée et praticité – elle supporte parfaitement le lavage en machine et conserve son éclat saison après saison, devenant vite un indispensable de votre dressing.</v>
       </c>
     </row>
-    <row r="24" ht="50" customHeight="1" spans="1:67">
+    <row r="24" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A24" s="4" t="s">
         <v>286</v>
       </c>
@@ -8712,15 +8720,15 @@
         <v>229</v>
       </c>
       <c r="D24" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
+      </c>
+      <c r="E24" s="4" t="str">
+        <f t="shared" si="20"/>
+        <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
+      </c>
+      <c r="F24" s="4">
         <f t="shared" si="18"/>
-        <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
-      </c>
-      <c r="E24" s="4" t="str">
-        <f t="shared" si="19"/>
-        <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
-      </c>
-      <c r="F24" s="4">
-        <f t="shared" si="17"/>
         <v>105</v>
       </c>
       <c r="G24" s="4"/>
@@ -8829,67 +8837,67 @@
         <v>24.66</v>
       </c>
       <c r="AY24" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>Col rabattu</v>
       </c>
       <c r="AZ24" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>Décontracté</v>
       </c>
       <c r="BA24" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>Occidental</v>
       </c>
       <c r="BB24" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>Chemise</v>
       </c>
       <c r="BC24" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>Régulier</v>
       </c>
       <c r="BD24" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>Plaine</v>
       </c>
       <c r="BE24" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>Col cranté</v>
       </c>
       <c r="BG24" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>Manches longues</v>
       </c>
       <c r="BH24" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>Manchette</v>
       </c>
       <c r="BI24" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>Bouton</v>
       </c>
       <c r="BK24" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>Tissu ultra-légèrement aéré : grâce à une sélection de matières premières nobles, nos chemises homme offrent une respirabilité exceptionnelle qui vous enveloppe d’une sensation de fraîcheur tout au long de la journée.</v>
       </c>
       <c r="BL24" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>Coupe moderne et intemporelle : ce modèle au design épuré mêle avec subtilité l’esprit classique et une touche contemporaine, pour un rendu aussi chic que décontracté, parfait pour vos journées estivales.</v>
       </c>
       <c r="BM24" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>Adaptée à toutes les situations : que vous flâniez en bord de mer, que vous participiez à un pique-nique entre amis ou que vous profitiez d’un moment de farniente à la maison, cette chemise en lin à manches longues s’impose comme la pièce maîtresse de vos tenues décontractées.</v>
       </c>
       <c r="BN24" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>Associations faciles et infinies : portez-la avec un bermuda, un pantalon en toile ou un jean brut, et vous obtiendrez en un clin d’œil une allure élégante et naturelle, qui passe sans effort de la lumière du jour aux soirées douces.</v>
       </c>
       <c r="BO24" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>Solidité et entretien simplifié : confectionnée selon un savoir-faire rigoureux, cette chemise d’été allie esthétique raffinée et praticité – elle supporte parfaitement le lavage en machine et conserve son éclat saison après saison, devenant vite un indispensable de votre dressing.</v>
       </c>
     </row>
-    <row r="25" ht="50" customHeight="1" spans="1:67">
+    <row r="25" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A25" s="4" t="s">
         <v>296</v>
       </c>
@@ -8900,15 +8908,15 @@
         <v>229</v>
       </c>
       <c r="D25" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
+      </c>
+      <c r="E25" s="4" t="str">
+        <f t="shared" si="20"/>
+        <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
+      </c>
+      <c r="F25" s="4">
         <f t="shared" si="18"/>
-        <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
-      </c>
-      <c r="E25" s="4" t="str">
-        <f t="shared" si="19"/>
-        <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
-      </c>
-      <c r="F25" s="4">
-        <f t="shared" si="17"/>
         <v>105</v>
       </c>
       <c r="G25" s="4"/>
@@ -9017,67 +9025,67 @@
         <v>24.56</v>
       </c>
       <c r="AY25" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>Col rabattu</v>
       </c>
       <c r="AZ25" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>Décontracté</v>
       </c>
       <c r="BA25" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>Occidental</v>
       </c>
       <c r="BB25" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>Chemise</v>
       </c>
       <c r="BC25" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>Régulier</v>
       </c>
       <c r="BD25" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>Plaine</v>
       </c>
       <c r="BE25" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>Col cranté</v>
       </c>
       <c r="BG25" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>Manches longues</v>
       </c>
       <c r="BH25" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>Manchette</v>
       </c>
       <c r="BI25" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>Bouton</v>
       </c>
       <c r="BK25" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>Tissu ultra-légèrement aéré : grâce à une sélection de matières premières nobles, nos chemises homme offrent une respirabilité exceptionnelle qui vous enveloppe d’une sensation de fraîcheur tout au long de la journée.</v>
       </c>
       <c r="BL25" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>Coupe moderne et intemporelle : ce modèle au design épuré mêle avec subtilité l’esprit classique et une touche contemporaine, pour un rendu aussi chic que décontracté, parfait pour vos journées estivales.</v>
       </c>
       <c r="BM25" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>Adaptée à toutes les situations : que vous flâniez en bord de mer, que vous participiez à un pique-nique entre amis ou que vous profitiez d’un moment de farniente à la maison, cette chemise en lin à manches longues s’impose comme la pièce maîtresse de vos tenues décontractées.</v>
       </c>
       <c r="BN25" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>Associations faciles et infinies : portez-la avec un bermuda, un pantalon en toile ou un jean brut, et vous obtiendrez en un clin d’œil une allure élégante et naturelle, qui passe sans effort de la lumière du jour aux soirées douces.</v>
       </c>
       <c r="BO25" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>Solidité et entretien simplifié : confectionnée selon un savoir-faire rigoureux, cette chemise d’été allie esthétique raffinée et praticité – elle supporte parfaitement le lavage en machine et conserve son éclat saison après saison, devenant vite un indispensable de votre dressing.</v>
       </c>
     </row>
-    <row r="26" ht="50" customHeight="1" spans="1:67">
+    <row r="26" ht="50" hidden="1" customHeight="1" spans="1:67">
       <c r="A26" s="4" t="s">
         <v>305</v>
       </c>
@@ -9088,15 +9096,15 @@
         <v>229</v>
       </c>
       <c r="D26" s="4" t="str">
+        <f t="shared" si="19"/>
+        <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
+      </c>
+      <c r="E26" s="4" t="str">
+        <f t="shared" si="20"/>
+        <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
+      </c>
+      <c r="F26" s="4">
         <f t="shared" si="18"/>
-        <v>Chemise Western Homme Imprimé Vintage Manches Longues</v>
-      </c>
-      <c r="E26" s="4" t="str">
-        <f t="shared" si="19"/>
-        <v>Géométrique Col Revers Boutonnage, Deux Poches Poitrine Plein Air, Western Décontracté Chemise Doux Lisse</v>
-      </c>
-      <c r="F26" s="4">
-        <f t="shared" si="17"/>
         <v>105</v>
       </c>
       <c r="G26" s="4"/>
@@ -9205,67 +9213,73 @@
         <v>24.84</v>
       </c>
       <c r="AY26" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>Col rabattu</v>
       </c>
       <c r="AZ26" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>Décontracté</v>
       </c>
       <c r="BA26" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>Occidental</v>
       </c>
       <c r="BB26" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>Chemise</v>
       </c>
       <c r="BC26" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>Régulier</v>
       </c>
       <c r="BD26" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>Plaine</v>
       </c>
       <c r="BE26" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>Col cranté</v>
       </c>
       <c r="BG26" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>Manches longues</v>
       </c>
       <c r="BH26" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>Manchette</v>
       </c>
       <c r="BI26" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>Bouton</v>
       </c>
       <c r="BK26" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>Tissu ultra-légèrement aéré : grâce à une sélection de matières premières nobles, nos chemises homme offrent une respirabilité exceptionnelle qui vous enveloppe d’une sensation de fraîcheur tout au long de la journée.</v>
       </c>
       <c r="BL26" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>Coupe moderne et intemporelle : ce modèle au design épuré mêle avec subtilité l’esprit classique et une touche contemporaine, pour un rendu aussi chic que décontracté, parfait pour vos journées estivales.</v>
       </c>
       <c r="BM26" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>Adaptée à toutes les situations : que vous flâniez en bord de mer, que vous participiez à un pique-nique entre amis ou que vous profitiez d’un moment de farniente à la maison, cette chemise en lin à manches longues s’impose comme la pièce maîtresse de vos tenues décontractées.</v>
       </c>
       <c r="BN26" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>Associations faciles et infinies : portez-la avec un bermuda, un pantalon en toile ou un jean brut, et vous obtiendrez en un clin d’œil une allure élégante et naturelle, qui passe sans effort de la lumière du jour aux soirées douces.</v>
       </c>
       <c r="BO26" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>Solidité et entretien simplifié : confectionnée selon un savoir-faire rigoureux, cette chemise d’été allie esthétique raffinée et praticité – elle supporte parfaitement le lavage en machine et conserve son éclat saison après saison, devenant vite un indispensable de votre dressing.</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:F26" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="0">
+      <colorFilter dxfId="0"/>
+    </filterColumn>
+    <extLst/>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <drawing r:id="rId1"/>

</xml_diff>